<commit_message>
v1.9.0: Revenue can be typed in
Revenue was calculated only. It is now a field. Blank means it follows the
prices as before, sale less purchase less repairs, or the fee on an
assignment. A typed figure stands regardless of what the prices do, and
clearing the box hands it back to the calculation.

The line under the box names which one is on screen, and when a typed figure
disagrees with the prices it says what they work out to, so the two cannot
quietly diverge. The board row shows whichever the property is using.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PD4vD51siFq5jYyNjR6B3w
</commit_message>
<xml_diff>
--- a/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
+++ b/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
@@ -534,12 +534,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -624,12 +624,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -665,12 +665,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -706,12 +706,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -747,12 +747,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -788,12 +788,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -829,12 +829,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -870,12 +870,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -911,12 +911,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -952,12 +952,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -993,12 +993,12 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -1075,12 +1075,12 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -1116,12 +1116,12 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -1157,12 +1157,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -1198,12 +1198,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -1239,12 +1239,12 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -1280,12 +1280,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -1321,12 +1321,12 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -1444,12 +1444,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH2"/>
+  <dimension ref="A1:AI2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1722,6 +1722,7 @@
     <col width="14" customWidth="1" min="32" max="32"/>
     <col width="16" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="14" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1893,6 +1894,11 @@
       <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>assignment_fee</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>revenue</t>
         </is>
       </c>
     </row>
@@ -1931,6 +1937,7 @@
       <c r="AF2" s="2" t="n"/>
       <c r="AG2" s="2" t="n"/>
       <c r="AH2" s="2" t="n"/>
+      <c r="AI2" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2490,12 +2497,12 @@
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S2" s="2" t="n"/>
@@ -2551,12 +2558,12 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S3" s="2" t="n"/>
@@ -2616,12 +2623,12 @@
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S4" s="2" t="n"/>
@@ -2681,12 +2688,12 @@
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S5" s="2" t="n"/>
@@ -2742,12 +2749,12 @@
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S6" s="2" t="n"/>
@@ -2803,12 +2810,12 @@
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S7" s="2" t="n"/>
@@ -2864,12 +2871,12 @@
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S8" s="2" t="n"/>
@@ -2925,12 +2932,12 @@
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S9" s="2" t="n"/>
@@ -2986,12 +2993,12 @@
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S10" s="2" t="n"/>
@@ -3047,12 +3054,12 @@
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S11" s="2" t="n"/>
@@ -3108,12 +3115,12 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S12" s="2" t="n"/>
@@ -3169,12 +3176,12 @@
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S13" s="2" t="n"/>
@@ -3230,12 +3237,12 @@
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S14" s="2" t="n"/>
@@ -3291,12 +3298,12 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S15" s="2" t="n"/>
@@ -3352,12 +3359,12 @@
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S16" s="2" t="n"/>
@@ -3413,12 +3420,12 @@
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S17" s="2" t="n"/>
@@ -3474,12 +3481,12 @@
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S18" s="2" t="n"/>
@@ -3535,12 +3542,12 @@
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S19" s="2" t="n"/>
@@ -3596,12 +3603,12 @@
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S20" s="2" t="n"/>
@@ -3657,12 +3664,12 @@
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S21" s="2" t="n"/>
@@ -3718,12 +3725,12 @@
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S22" s="2" t="n"/>
@@ -3779,12 +3786,12 @@
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
       <c r="S23" s="2" t="n"/>
@@ -3994,7 +4001,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -4016,7 +4023,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -4038,7 +4045,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -4060,7 +4067,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -4082,7 +4089,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4111,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -4116,7 +4123,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1.7.0</t>
+          <t>1.9.0</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -4126,7 +4133,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -4148,7 +4155,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4177,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -4192,7 +4199,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>
@@ -4214,7 +4221,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:20:23.000Z</t>
+          <t>2026-09-14T15:22:24.000Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v1.9.2: add contract cancelled as an archive outcome
A contract that dies had nowhere accurate to go: sold, no equity, not
interested and bad data all describe a lead that never got that far.

Archived: contract cancelled is now its own outcome, first in the archive
list because it is the one that cost us something. It lands on the Archived
tab rather than Closed, is counted by name in the pipeline's archived-by-
reason breakdown, and restores to Under contract if the seller returns.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PD4vD51siFq5jYyNjR6B3w
</commit_message>
<xml_diff>
--- a/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
+++ b/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
@@ -534,12 +534,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -624,12 +624,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -665,12 +665,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -706,12 +706,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -747,12 +747,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -788,12 +788,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -829,12 +829,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -870,12 +870,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -911,12 +911,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -952,12 +952,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -993,12 +993,12 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -1075,12 +1075,12 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -1116,12 +1116,12 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -1157,12 +1157,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -1198,12 +1198,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -1239,12 +1239,12 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -1280,12 +1280,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -1321,12 +1321,12 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -1444,12 +1444,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -2497,12 +2497,12 @@
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S2" s="2" t="n"/>
@@ -2558,12 +2558,12 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S3" s="2" t="n"/>
@@ -2623,12 +2623,12 @@
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S4" s="2" t="n"/>
@@ -2688,12 +2688,12 @@
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S5" s="2" t="n"/>
@@ -2749,12 +2749,12 @@
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S6" s="2" t="n"/>
@@ -2810,12 +2810,12 @@
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S7" s="2" t="n"/>
@@ -2871,12 +2871,12 @@
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S8" s="2" t="n"/>
@@ -2932,12 +2932,12 @@
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S9" s="2" t="n"/>
@@ -2993,12 +2993,12 @@
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S10" s="2" t="n"/>
@@ -3054,12 +3054,12 @@
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S11" s="2" t="n"/>
@@ -3115,12 +3115,12 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S12" s="2" t="n"/>
@@ -3176,12 +3176,12 @@
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S13" s="2" t="n"/>
@@ -3237,12 +3237,12 @@
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S14" s="2" t="n"/>
@@ -3298,12 +3298,12 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S15" s="2" t="n"/>
@@ -3359,12 +3359,12 @@
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S16" s="2" t="n"/>
@@ -3420,12 +3420,12 @@
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S17" s="2" t="n"/>
@@ -3481,12 +3481,12 @@
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S18" s="2" t="n"/>
@@ -3542,12 +3542,12 @@
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S19" s="2" t="n"/>
@@ -3603,12 +3603,12 @@
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S20" s="2" t="n"/>
@@ -3664,12 +3664,12 @@
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S21" s="2" t="n"/>
@@ -3725,12 +3725,12 @@
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S22" s="2" t="n"/>
@@ -3786,12 +3786,12 @@
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
       <c r="S23" s="2" t="n"/>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -4045,7 +4045,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -4089,7 +4089,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -4123,7 +4123,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1.9.0</t>
+          <t>1.9.2</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -4155,7 +4155,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -4177,7 +4177,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:22:24.000Z</t>
+          <t>2026-09-15T15:14:56.000Z</t>
         </is>
       </c>
     </row>

</xml_diff>